<commit_message>
fix: remove unused imports
fix: remove unused imports
</commit_message>
<xml_diff>
--- a/backend/inquiries.xlsx
+++ b/backend/inquiries.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -819,9 +819,44 @@
         <v>New</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13">
+        <v>1788442585076</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Jaysinh Parmar</v>
+      </c>
+      <c r="C13" t="str">
+        <v>56546</v>
+      </c>
+      <c r="D13" t="str">
+        <v>jaysinhparmar7777@gmail.com</v>
+      </c>
+      <c r="E13" t="str">
+        <v>07203064555</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Kitchenware</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Containers</v>
+      </c>
+      <c r="H13" t="str">
+        <v>50</v>
+      </c>
+      <c r="I13" t="str">
+        <v>lkl</v>
+      </c>
+      <c r="J13" t="str">
+        <v>2026-09-03T13:36:25.076Z</v>
+      </c>
+      <c r="K13" t="str">
+        <v>New</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>